<commit_message>
Add iPLA calibrator evaluation notebook with publication figure
</commit_message>
<xml_diff>
--- a/ELISA Ab SNR/SNR_Hytest.xlsx
+++ b/ELISA Ab SNR/SNR_Hytest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wehieduau-my.sharepoint.com/personal/smith_j_wehi_edu_au/Documents/Documents/CFHAC_ProxiPal/ProxiPal/user_documents/NfL-PLA Development Paper/NfL-PLA Development Paper Figure Data/a_ELISA Antibody Performance_waiting data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wehieduau-my.sharepoint.com/personal/smith_j_wehi_edu_au/Documents/Documents/CFHAC_ProxiPal/ProxiPal/user_documents/NfL-PLA Development Paper/NfL-PLA Development Paper Figure Data/GitHub/NfL-iPLA-paper/ELISA Ab SNR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{DE0DB712-E645-4E65-8640-DEA8352687B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E00C3DEF-E8E5-4435-8737-69D667ED36A8}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{DE0DB712-E645-4E65-8640-DEA8352687B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18C360B3-BBDD-4D8E-A643-33382C4485D3}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="1980" windowWidth="30810" windowHeight="19620" activeTab="1" xr2:uid="{5D19D104-DE1A-4A89-B45D-55E73A3C36C1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{5D19D104-DE1A-4A89-B45D-55E73A3C36C1}"/>
   </bookViews>
   <sheets>
     <sheet name="SNR_Hytest" sheetId="1" r:id="rId1"/>
@@ -645,10 +645,10 @@
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1771,7 +1771,7 @@
       </c>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -1809,20 +1809,20 @@
       </c>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="9"/>
+      <c r="B5" s="10"/>
       <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="9">
         <v>17.899999999999999</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="9">
         <v>16.3</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="9">
         <v>17.8</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="9">
         <v>19.8</v>
       </c>
       <c r="H5" s="5">
@@ -1931,7 +1931,7 @@
       </c>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="4" t="s">
@@ -1969,7 +1969,7 @@
       </c>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="9"/>
+      <c r="B10" s="10"/>
       <c r="C10" s="4" t="s">
         <v>14</v>
       </c>
@@ -2091,7 +2091,7 @@
       </c>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="10" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="4" t="s">
@@ -2129,7 +2129,7 @@
       </c>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B15" s="9"/>
+      <c r="B15" s="10"/>
       <c r="C15" s="4" t="s">
         <v>14</v>
       </c>
@@ -2251,7 +2251,7 @@
       </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="10" t="s">
         <v>15</v>
       </c>
       <c r="C19" s="4" t="s">
@@ -2289,20 +2289,20 @@
       </c>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B20" s="9"/>
+      <c r="B20" s="10"/>
       <c r="C20" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="10">
+      <c r="D20" s="9">
         <v>22</v>
       </c>
-      <c r="E20" s="10">
+      <c r="E20" s="9">
         <v>21.1</v>
       </c>
-      <c r="F20" s="10">
+      <c r="F20" s="9">
         <v>22.5</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="9">
         <v>25.2</v>
       </c>
       <c r="H20" s="5">
@@ -2460,7 +2460,9 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="27" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>